<commit_message>
Replace 図鑑番号 with a per-刀剣男士 number
- Rename the Excel column to 刀剣男士番号; all costume / rare variants
  of the same 刀剣男士 share one number (三日月宗近 レア: 4 -> 3)
- Warn when one 刀剣男士 has different numbers or one number is used by
  different 刀剣男士
- Converter prefers exact header matches so 刀剣男士 does not pick up
  the 刀剣男士番号 column

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmcWsZyXqCtsLFgw44gTJT
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -473,7 +473,7 @@
     <row r="1">
       <c r="A1" s="0" t="inlineStr">
         <is>
-          <t>刀図鑑</t>
+          <t>刀剣男士番号</t>
         </is>
       </c>
       <c r="B1" s="0" t="inlineStr">
@@ -481,12 +481,12 @@
           <t>刀剣男士</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>衣装</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>レア</t>
         </is>
@@ -551,7 +551,7 @@
           <t>三日月宗近</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>戦装束</t>
         </is>
@@ -559,19 +559,19 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
           <t>三日月宗近</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>戦装束</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>○</t>
         </is>
@@ -586,7 +586,7 @@
           <t>小狐丸</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>戦装束</t>
         </is>
@@ -606,7 +606,7 @@
           <t>石切丸</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>戦装束</t>
         </is>

</xml_diff>

<commit_message>
Add second batch of character data from screenshots
骨喰藤四郎, 三日月宗近（レア, 奥義名 only; 13lv 1060,140 confirmed by
the screenshot）, 一期一振, 乱藤四郎 and 山姥切国広.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmcWsZyXqCtsLFgw44gTJT
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -820,6 +820,11 @@
       <c r="H3" t="n">
         <v>22</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>月明かりの冴え</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>【すべて】のト餓鬼を消去し、敵に【特小++】ダメージを与える</t>
@@ -1132,6 +1137,29 @@
           <t>太刀</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>兄弟</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>黄</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>22</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>水平一刀斬り</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>【横列・小範囲】のト餓鬼を消去し、敵に【特小＋＋】ダメージを与える</t>
+        </is>
+      </c>
       <c r="O8" s="1" t="n"/>
       <c r="P8" s="1" t="n"/>
       <c r="Q8" s="1" t="n"/>
@@ -1142,7 +1170,11 @@
       <c r="V8" s="1" t="n"/>
       <c r="W8" s="1" t="n"/>
       <c r="X8" s="1" t="n"/>
-      <c r="Y8" s="1" t="n"/>
+      <c r="Y8" s="1" t="inlineStr">
+        <is>
+          <t>1050,108</t>
+        </is>
+      </c>
       <c r="Z8" s="1" t="n"/>
       <c r="AA8" s="1" t="n"/>
       <c r="AB8" s="1" t="n"/>
@@ -1320,6 +1352,29 @@
           <t>脇差</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>兄弟</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>黄</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>14</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>色変幻の術・青</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>青以外のト餓鬼を【最大10体】、青色に変換する</t>
+        </is>
+      </c>
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="n"/>
       <c r="Q11" s="1" t="n"/>
@@ -1335,7 +1390,11 @@
       <c r="AA11" s="1" t="n"/>
       <c r="AB11" s="1" t="n"/>
       <c r="AC11" s="1" t="n"/>
-      <c r="AD11" s="1" t="n"/>
+      <c r="AD11" s="1" t="inlineStr">
+        <is>
+          <t>1024,163</t>
+        </is>
+      </c>
       <c r="AE11" s="1" t="n"/>
       <c r="AF11" s="1" t="n"/>
       <c r="AG11" s="1" t="n"/>
@@ -1506,6 +1565,29 @@
           <t>短刀</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>兄弟</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>黄</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>12</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>色変幻の術・乱</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>ト餓鬼を【最大10体】、ランダムな色に変換する</t>
+        </is>
+      </c>
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="n"/>
       <c r="Q14" s="1" t="n"/>
@@ -1515,7 +1597,11 @@
       <c r="U14" s="1" t="n"/>
       <c r="V14" s="1" t="n"/>
       <c r="W14" s="1" t="n"/>
-      <c r="X14" s="1" t="n"/>
+      <c r="X14" s="1" t="inlineStr">
+        <is>
+          <t>905,100</t>
+        </is>
+      </c>
       <c r="Y14" s="1" t="n"/>
       <c r="Z14" s="1" t="n"/>
       <c r="AA14" s="1" t="n"/>
@@ -1909,6 +1995,29 @@
           <t>打刀</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>兄弟</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>青</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>22</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>正円一刀斬り</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>【円型・小範囲】のト餓鬼を消去し、敵に【小】ダメージを与える</t>
+        </is>
+      </c>
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="n"/>
       <c r="Q23" s="1" t="n"/>
@@ -1918,7 +2027,11 @@
       <c r="U23" s="1" t="n"/>
       <c r="V23" s="1" t="n"/>
       <c r="W23" s="1" t="n"/>
-      <c r="X23" s="1" t="n"/>
+      <c r="X23" s="1" t="inlineStr">
+        <is>
+          <t>850,107</t>
+        </is>
+      </c>
       <c r="Y23" s="1" t="n"/>
       <c r="Z23" s="1" t="n"/>
       <c r="AA23" s="1" t="n"/>

</xml_diff>

<commit_message>
Add third batch of character data from screenshots
鶴丸国永, 蛍丸, 小狐丸 (奥義名 added; existing values confirmed), 加州清光
and 獅子王.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmcWsZyXqCtsLFgw44gTJT
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -900,6 +900,11 @@
       <c r="H4" t="n">
         <v>27</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ボム練成の術 三の火</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>ボムを【3個】生成する</t>
@@ -909,7 +914,7 @@
       <c r="P4" s="1" t="n"/>
       <c r="Q4" s="1" t="n"/>
       <c r="R4" s="1" t="n"/>
-      <c r="S4" s="6" t="inlineStr">
+      <c r="S4" s="1" t="inlineStr">
         <is>
           <t>740,77</t>
         </is>
@@ -1723,6 +1728,34 @@
           <t>大太刀</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>夜</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>青</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>36</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>正円一刀斬り</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>【円型・大範囲】のト餓鬼を消去し、敵に【中＋】ダメージを与える</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>677,107</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1781,13 +1814,40 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>打刀</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>新選組</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>赤</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>26</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>必中三段斬り</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>指定した【円型・特小範囲】のト餓鬼を3回消去し、敵に【小】ダメージを与える</t>
         </is>
       </c>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="n"/>
       <c r="Q20" s="1" t="n"/>
       <c r="R20" s="1" t="n"/>
-      <c r="S20" s="1" t="n"/>
+      <c r="S20" s="1" t="inlineStr">
+        <is>
+          <t>645,73</t>
+        </is>
+      </c>
       <c r="T20" s="1" t="n"/>
       <c r="U20" s="1" t="n"/>
       <c r="V20" s="1" t="n"/>
@@ -2128,11 +2188,38 @@
           <t>太刀</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>けもの</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>赤</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>22</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>水平一刀斬り</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>【横列・小範囲】のト餓鬼を消去し、敵に【小＋】ダメージを与える</t>
+        </is>
+      </c>
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="n"/>
       <c r="Q25" s="1" t="n"/>
       <c r="R25" s="1" t="n"/>
-      <c r="S25" s="1" t="n"/>
+      <c r="S25" s="1" t="inlineStr">
+        <is>
+          <t>771,74</t>
+        </is>
+      </c>
       <c r="T25" s="1" t="n"/>
       <c r="U25" s="1" t="n"/>
       <c r="V25" s="1" t="n"/>
@@ -2181,6 +2268,30 @@
           <t>太刀</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>鳥</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>赤</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>24</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>水平斬り 攻勢の型</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>【横列・中範囲】のト餓鬼を消去し、敵に【小＋】ダメージを与える
+自身に攻撃力上昇【極小・1手】を付与する</t>
+        </is>
+      </c>
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="n"/>
       <c r="Q26" s="1" t="n"/>
@@ -2190,7 +2301,11 @@
       <c r="U26" s="1" t="n"/>
       <c r="V26" s="1" t="n"/>
       <c r="W26" s="1" t="n"/>
-      <c r="X26" s="1" t="n"/>
+      <c r="X26" s="1" t="inlineStr">
+        <is>
+          <t>935,110</t>
+        </is>
+      </c>
       <c r="Y26" s="1" t="n"/>
       <c r="Z26" s="1" t="n"/>
       <c r="AA26" s="1" t="n"/>

</xml_diff>

<commit_message>
Add fourth batch of character data from screenshots
石切丸 (奥義名; 奥義 text updated to the in-game wording 味方全員に), 岩融,
厚藤四郎, 五虎退 and 蜻蛉切.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmcWsZyXqCtsLFgw44gTJT
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -980,12 +980,18 @@
       <c r="H5" t="n">
         <v>22</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>逆さ扇斬り 守護の型</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>【扇型・中範囲】のト餓鬼を消去し、敵に【特小-】ダメージを与える。味方全体に被ダメージ軽減【極小+・3手】を付与する</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
+          <t>【扇型・中範囲】のト餓鬼を消去し、敵に【特小－】ダメージを与える。
+味方全員に被ダメージ軽減【極小＋・3手】を付与する</t>
+        </is>
+      </c>
+      <c r="O5" s="1" t="inlineStr">
         <is>
           <t>561,61</t>
         </is>
@@ -1042,6 +1048,34 @@
           <t>薙刀</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>源氏</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>青</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>大薙ぎ払い・赤</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>【最大10体】の赤ト餓鬼を盤面の右下に集める</t>
+        </is>
+      </c>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>471,69</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1517,7 +1551,34 @@
           <t>短刀</t>
         </is>
       </c>
-      <c r="O13" s="1" t="n"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>兄弟</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>黄</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>色変幻の術・青</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>赤色のト餓鬼を【最大10体】、青色に変換する</t>
+        </is>
+      </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>440,77</t>
+        </is>
+      </c>
       <c r="P13" s="1" t="n"/>
       <c r="Q13" s="1" t="n"/>
       <c r="R13" s="1" t="n"/>
@@ -1675,7 +1736,34 @@
           <t>短刀</t>
         </is>
       </c>
-      <c r="O16" s="1" t="n"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>兄弟</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>赤</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>13</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>ボム練成の術 一の火</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>ボムを【1個】生成する</t>
+        </is>
+      </c>
+      <c r="O16" s="1" t="inlineStr">
+        <is>
+          <t>477,56</t>
+        </is>
+      </c>
       <c r="P16" s="1" t="n"/>
       <c r="Q16" s="1" t="n"/>
       <c r="R16" s="1" t="n"/>
@@ -1774,6 +1862,34 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>槍</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>天下三名槍</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>黄</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>22</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>必中縦断突き</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>指定した【縦列・小範囲】のト餓鬼を消去し、敵に【小】ダメージを与える</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>551,72</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 江雪左文字 and 山伏国広 data from screenshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmcWsZyXqCtsLFgw44gTJT
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -1912,6 +1912,35 @@
           <t>太刀</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>雪</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>赤</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>19</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>霧散斬り 先手の型</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>ランダムなト餓鬼（攻撃指示優先）を最大5体消去し、敵に【特小＋＋】ダメージを与える
+消去時のブレイクゲージ減少量が【2倍】になる</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>507,74</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2251,7 +2280,35 @@
           <t>太刀</t>
         </is>
       </c>
-      <c r="O24" s="1" t="n"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>お山修行</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>赤</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>22</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>逆さ扇斬り 守護の型</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>【扇型・特小範囲】のト餓鬼を消去し、敵に【極小＋】ダメージを与える
+味方全員に被ダメージ軽減【特小＋＋・3手】を付与する</t>
+        </is>
+      </c>
+      <c r="O24" s="1" t="inlineStr">
+        <is>
+          <t>584,70</t>
+        </is>
+      </c>
       <c r="P24" s="1" t="n"/>
       <c r="Q24" s="1" t="n"/>
       <c r="R24" s="1" t="n"/>

</xml_diff>

<commit_message>
Add 陸奥守吉行 奥義名 from screenshot; match 奥義 text to the game
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FmcWsZyXqCtsLFgw44gTJT
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -2134,9 +2134,15 @@
       <c r="H22" t="n">
         <v>16</v>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>水平斬り 攻勢の型</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>【横列・小範囲】のト餓鬼を消去し、敵に【極小】ダメージを与える味方全員に攻撃力上昇【極小++・3手】を付与する</t>
+          <t>【横列・小範囲】のト餓鬼を消去し、敵に【極小】ダメージを与える
+味方全員に攻撃力上昇【極小＋＋・3手】を付与する</t>
         </is>
       </c>
       <c r="O22" s="1" t="n"/>

</xml_diff>